<commit_message>
Update 1/2 after paper acceptance
</commit_message>
<xml_diff>
--- a/SNA_matrix.xlsx
+++ b/SNA_matrix.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cnrsc-my.sharepoint.com/personal/roberto_malvezzi_cnr_it/Documents/04_Universo post-traumatico/02_Survey Wellbeing/Publishing/Submission Urban Science/1st round Review/Excel per review Urban Science/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\EliaMTh\Desktop\SNAgraph\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="90" documentId="8_{E281E7CD-93E7-4F4A-A990-59692DAED7D0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3F59D46C-F8E0-4784-85ED-804B30B615DE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DCBFFFEE-6C32-4A08-9AFA-4437168DCFB2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" activeTab="3" xr2:uid="{68C387C8-9578-49CC-B16D-AB3062C06B27}"/>
+    <workbookView xWindow="780" yWindow="780" windowWidth="28800" windowHeight="15435" xr2:uid="{68C387C8-9578-49CC-B16D-AB3062C06B27}"/>
   </bookViews>
   <sheets>
     <sheet name="Topics" sheetId="2" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="53">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="342" uniqueCount="51">
   <si>
     <t>Education</t>
   </si>
@@ -194,12 +194,6 @@
     <t>Mental Health and WB</t>
   </si>
   <si>
-    <t>peso</t>
-  </si>
-  <si>
-    <t>(da clusterizzazione)</t>
-  </si>
-  <si>
     <t>pesi</t>
   </si>
 </sst>
@@ -294,7 +288,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -311,9 +305,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="1" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -321,9 +312,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="center"/>
@@ -665,547 +653,394 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D674DE22-1809-43E4-BFE9-DA6D0B7C88B1}">
-  <dimension ref="A1:D49"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A2:B49"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="2" max="2" width="51.6640625" style="2" customWidth="1"/>
-    <col min="3" max="3" width="8.88671875" style="11"/>
+    <col min="2" max="2" width="51.7109375" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="C1" s="11" t="s">
-        <v>50</v>
-      </c>
-      <c r="D1" t="s">
-        <v>51</v>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" s="1">
+        <v>1</v>
+      </c>
+      <c r="B2" s="9" t="s">
+        <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="1">
-        <v>1</v>
-      </c>
-      <c r="B2" s="10" t="s">
-        <v>5</v>
-      </c>
-      <c r="C2" s="7">
-        <v>28</v>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A3" s="1">
+        <v>2</v>
+      </c>
+      <c r="B3" s="9" t="s">
+        <v>6</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="1">
-        <v>2</v>
-      </c>
-      <c r="B3" s="10" t="s">
-        <v>6</v>
-      </c>
-      <c r="C3" s="7">
-        <v>33</v>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A4" s="1">
+        <v>3</v>
+      </c>
+      <c r="B4" s="9" t="s">
+        <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="1">
-        <v>3</v>
-      </c>
-      <c r="B4" s="10" t="s">
-        <v>7</v>
-      </c>
-      <c r="C4" s="7">
-        <v>40</v>
-      </c>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A5" s="1">
         <v>4</v>
       </c>
-      <c r="B5" s="10" t="s">
+      <c r="B5" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="C5" s="7">
-        <v>22</v>
-      </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A6" s="1">
         <v>5</v>
       </c>
-      <c r="B6" s="10" t="s">
+      <c r="B6" s="9" t="s">
         <v>9</v>
       </c>
-      <c r="C6" s="7">
-        <v>12</v>
-      </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A7" s="1">
         <v>6</v>
       </c>
-      <c r="B7" s="10" t="s">
+      <c r="B7" s="9" t="s">
         <v>10</v>
       </c>
-      <c r="C7" s="7">
-        <v>24</v>
-      </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A8" s="1">
         <v>7</v>
       </c>
-      <c r="B8" s="10" t="s">
+      <c r="B8" s="9" t="s">
         <v>11</v>
       </c>
-      <c r="C8" s="7">
-        <v>12</v>
-      </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A9" s="1">
         <v>8</v>
       </c>
-      <c r="B9" s="10" t="s">
+      <c r="B9" s="9" t="s">
         <v>12</v>
       </c>
-      <c r="C9" s="7">
-        <v>33</v>
-      </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A10" s="1">
         <v>9</v>
       </c>
-      <c r="B10" s="10" t="s">
+      <c r="B10" s="9" t="s">
         <v>13</v>
       </c>
-      <c r="C10" s="7">
-        <v>12</v>
-      </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A11" s="1">
         <v>10</v>
       </c>
-      <c r="B11" s="10" t="s">
+      <c r="B11" s="9" t="s">
         <v>14</v>
       </c>
-      <c r="C11" s="7">
-        <v>27</v>
-      </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A12" s="1">
         <v>11</v>
       </c>
-      <c r="B12" s="10" t="s">
-        <v>0</v>
-      </c>
-      <c r="C12" s="7">
-        <v>14</v>
+      <c r="B12" s="9" t="s">
+        <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A13" s="1">
         <v>12</v>
       </c>
-      <c r="B13" s="10" t="s">
+      <c r="B13" s="9" t="s">
         <v>15</v>
       </c>
-      <c r="C13" s="7">
-        <v>24</v>
-      </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A14" s="1">
         <v>13</v>
       </c>
-      <c r="B14" s="10" t="s">
+      <c r="B14" s="9" t="s">
         <v>16</v>
       </c>
-      <c r="C14" s="7">
-        <v>20</v>
-      </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A15" s="1">
         <v>14</v>
       </c>
-      <c r="B15" s="10" t="s">
+      <c r="B15" s="9" t="s">
         <v>17</v>
       </c>
-      <c r="C15" s="7">
-        <v>16</v>
-      </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A16" s="1">
         <v>15</v>
       </c>
-      <c r="B16" s="10" t="s">
+      <c r="B16" s="9" t="s">
         <v>18</v>
       </c>
-      <c r="C16" s="7">
-        <v>15</v>
-      </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A17" s="1">
         <v>16</v>
       </c>
-      <c r="B17" s="10" t="s">
+      <c r="B17" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="C17" s="7">
-        <v>21</v>
-      </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A18" s="1">
         <v>17</v>
       </c>
-      <c r="B18" s="10" t="s">
+      <c r="B18" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="C18" s="7">
-        <v>65</v>
-      </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A19" s="1">
         <v>18</v>
       </c>
-      <c r="B19" s="10" t="s">
+      <c r="B19" s="9" t="s">
         <v>21</v>
       </c>
-      <c r="C19" s="7">
-        <v>39</v>
-      </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A20" s="1">
         <v>19</v>
       </c>
-      <c r="B20" s="10" t="s">
+      <c r="B20" s="9" t="s">
         <v>22</v>
       </c>
-      <c r="C20" s="7">
-        <v>10</v>
-      </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A21" s="1">
         <v>20</v>
       </c>
-      <c r="B21" s="10" t="s">
+      <c r="B21" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="C21" s="7">
-        <v>27</v>
-      </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A22" s="1">
         <v>21</v>
       </c>
-      <c r="B22" s="10" t="s">
+      <c r="B22" s="9" t="s">
         <v>24</v>
       </c>
-      <c r="C22" s="7">
-        <v>21</v>
-      </c>
     </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A23" s="1">
         <v>22</v>
       </c>
-      <c r="B23" s="10" t="s">
+      <c r="B23" s="9" t="s">
         <v>25</v>
       </c>
-      <c r="C23" s="7">
-        <v>22</v>
-      </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A24" s="1">
         <v>23</v>
       </c>
-      <c r="B24" s="10" t="s">
+      <c r="B24" s="9" t="s">
         <v>26</v>
       </c>
-      <c r="C24" s="7">
-        <v>32</v>
-      </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A25" s="1">
         <v>24</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B25" s="9" t="s">
         <v>27</v>
       </c>
-      <c r="C25" s="7">
-        <v>23</v>
-      </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A26" s="1">
         <v>25</v>
       </c>
-      <c r="B26" s="10" t="s">
+      <c r="B26" s="9" t="s">
         <v>28</v>
       </c>
-      <c r="C26" s="7">
-        <v>26</v>
-      </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A27" s="1">
         <v>26</v>
       </c>
-      <c r="B27" s="10" t="s">
-        <v>1</v>
-      </c>
-      <c r="C27" s="7">
-        <v>22</v>
+      <c r="B27" s="9" t="s">
+        <v>1</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A28" s="1">
         <v>27</v>
       </c>
-      <c r="B28" s="10" t="s">
+      <c r="B28" s="9" t="s">
         <v>29</v>
       </c>
-      <c r="C28" s="7">
-        <v>22</v>
-      </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A29" s="1">
         <v>28</v>
       </c>
-      <c r="B29" s="10" t="s">
+      <c r="B29" s="9" t="s">
         <v>30</v>
       </c>
-      <c r="C29" s="7">
-        <v>17</v>
-      </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A30" s="1">
         <v>29</v>
       </c>
-      <c r="B30" s="10" t="s">
+      <c r="B30" s="9" t="s">
         <v>31</v>
       </c>
-      <c r="C30" s="7">
-        <v>34</v>
-      </c>
     </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A31" s="1">
         <v>30</v>
       </c>
-      <c r="B31" s="10" t="s">
+      <c r="B31" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="C31" s="7">
-        <v>11</v>
-      </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A32" s="1">
         <v>31</v>
       </c>
-      <c r="B32" s="10" t="s">
+      <c r="B32" s="9" t="s">
         <v>33</v>
       </c>
-      <c r="C32" s="7">
-        <v>21</v>
-      </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A33" s="1">
         <v>32</v>
       </c>
-      <c r="B33" s="10" t="s">
+      <c r="B33" s="9" t="s">
         <v>34</v>
       </c>
-      <c r="C33" s="7">
-        <v>28</v>
-      </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A34" s="1">
         <v>33</v>
       </c>
-      <c r="B34" s="10" t="s">
+      <c r="B34" s="9" t="s">
         <v>35</v>
       </c>
-      <c r="C34" s="7">
-        <v>38</v>
-      </c>
     </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A35" s="1">
         <v>34</v>
       </c>
-      <c r="B35" s="10" t="s">
+      <c r="B35" s="9" t="s">
         <v>36</v>
       </c>
-      <c r="C35" s="7">
-        <v>12</v>
-      </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A36" s="1">
         <v>35</v>
       </c>
-      <c r="B36" s="10" t="s">
+      <c r="B36" s="9" t="s">
         <v>37</v>
       </c>
-      <c r="C36" s="7">
-        <v>10</v>
-      </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A37" s="1">
         <v>36</v>
       </c>
-      <c r="B37" s="10" t="s">
-        <v>2</v>
-      </c>
-      <c r="C37" s="7">
-        <v>28</v>
+      <c r="B37" s="9" t="s">
+        <v>2</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A38" s="1">
         <v>37</v>
       </c>
-      <c r="B38" s="10" t="s">
+      <c r="B38" s="9" t="s">
         <v>38</v>
       </c>
-      <c r="C38" s="7">
-        <v>16</v>
-      </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A39" s="1">
         <v>38</v>
       </c>
-      <c r="B39" s="10" t="s">
+      <c r="B39" s="9" t="s">
         <v>39</v>
       </c>
-      <c r="C39" s="7">
-        <v>11</v>
-      </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A40" s="1">
         <v>39</v>
       </c>
-      <c r="B40" s="10" t="s">
+      <c r="B40" s="9" t="s">
         <v>40</v>
       </c>
-      <c r="C40" s="7">
-        <v>17</v>
-      </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A41" s="1">
         <v>40</v>
       </c>
-      <c r="B41" s="10" t="s">
+      <c r="B41" s="9" t="s">
         <v>41</v>
       </c>
-      <c r="C41" s="7">
-        <v>22</v>
-      </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A42" s="1">
         <v>41</v>
       </c>
-      <c r="B42" s="10" t="s">
+      <c r="B42" s="9" t="s">
         <v>42</v>
       </c>
-      <c r="C42" s="7">
-        <v>13</v>
-      </c>
     </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A43" s="1">
         <v>42</v>
       </c>
-      <c r="B43" s="10" t="s">
+      <c r="B43" s="9" t="s">
         <v>43</v>
       </c>
-      <c r="C43" s="7">
-        <v>10</v>
-      </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A44" s="1">
         <v>43</v>
       </c>
-      <c r="B44" s="10" t="s">
-        <v>3</v>
-      </c>
-      <c r="C44" s="7">
-        <v>21</v>
+      <c r="B44" s="9" t="s">
+        <v>3</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A45" s="1">
         <v>44</v>
       </c>
-      <c r="B45" s="10" t="s">
+      <c r="B45" s="9" t="s">
         <v>44</v>
       </c>
-      <c r="C45" s="7">
-        <v>25</v>
-      </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A46" s="1">
         <v>45</v>
       </c>
-      <c r="B46" s="10" t="s">
+      <c r="B46" s="9" t="s">
         <v>45</v>
       </c>
-      <c r="C46" s="7">
-        <v>22</v>
-      </c>
     </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A47" s="1">
         <v>46</v>
       </c>
-      <c r="B47" s="10" t="s">
+      <c r="B47" s="9" t="s">
         <v>46</v>
       </c>
-      <c r="C47" s="7">
-        <v>67</v>
-      </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A48" s="1">
         <v>47</v>
       </c>
-      <c r="B48" s="10" t="s">
+      <c r="B48" s="9" t="s">
         <v>4</v>
       </c>
-      <c r="C48" s="7">
-        <v>55</v>
-      </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A49" s="1">
         <v>48</v>
       </c>
-      <c r="B49" s="10" t="s">
+      <c r="B49" s="9" t="s">
         <v>47</v>
-      </c>
-      <c r="C49" s="7">
-        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -1216,12 +1051,12 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9A46B714-DFC6-40A1-A0B1-874A094C5245}">
   <dimension ref="A1:AX53"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.88671875" customWidth="1"/>
+    <col min="1" max="1" width="28.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>48</v>
       </c>
@@ -1370,7 +1205,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -1519,7 +1354,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
@@ -1668,7 +1503,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
@@ -1817,7 +1652,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -1966,7 +1801,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
@@ -2115,7 +1950,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -2264,7 +2099,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>11</v>
       </c>
@@ -2413,7 +2248,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -2562,7 +2397,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>13</v>
       </c>
@@ -2711,7 +2546,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
@@ -2860,7 +2695,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>0</v>
       </c>
@@ -3009,7 +2844,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>15</v>
       </c>
@@ -3158,7 +2993,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
@@ -3307,7 +3142,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
@@ -3456,7 +3291,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>18</v>
       </c>
@@ -3605,7 +3440,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
@@ -3754,7 +3589,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
@@ -3903,7 +3738,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="19" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>21</v>
       </c>
@@ -4052,7 +3887,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>22</v>
       </c>
@@ -4201,7 +4036,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>49</v>
       </c>
@@ -4350,7 +4185,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>24</v>
       </c>
@@ -4499,7 +4334,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>25</v>
       </c>
@@ -4648,7 +4483,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
@@ -4797,7 +4632,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="25" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>27</v>
       </c>
@@ -4946,7 +4781,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="26" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>28</v>
       </c>
@@ -5095,7 +4930,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>1</v>
       </c>
@@ -5244,7 +5079,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>29</v>
       </c>
@@ -5393,7 +5228,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>30</v>
       </c>
@@ -5542,7 +5377,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="30" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
@@ -5691,7 +5526,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="31" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>32</v>
       </c>
@@ -5840,7 +5675,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="32" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>33</v>
       </c>
@@ -5989,7 +5824,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="33" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>34</v>
       </c>
@@ -6138,7 +5973,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>35</v>
       </c>
@@ -6287,7 +6122,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="35" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>36</v>
       </c>
@@ -6436,7 +6271,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="36" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>37</v>
       </c>
@@ -6585,7 +6420,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="37" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>2</v>
       </c>
@@ -6734,7 +6569,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>38</v>
       </c>
@@ -6883,7 +6718,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>39</v>
       </c>
@@ -7032,7 +6867,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>40</v>
       </c>
@@ -7181,7 +7016,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>41</v>
       </c>
@@ -7330,7 +7165,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="42" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>42</v>
       </c>
@@ -7479,7 +7314,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="43" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>43</v>
       </c>
@@ -7628,7 +7463,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="44" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>3</v>
       </c>
@@ -7777,7 +7612,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>44</v>
       </c>
@@ -7926,7 +7761,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="46" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>45</v>
       </c>
@@ -8075,7 +7910,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>46</v>
       </c>
@@ -8224,7 +8059,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="48" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>4</v>
       </c>
@@ -8373,7 +8208,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:50" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:50" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>47</v>
       </c>
@@ -8522,152 +8357,152 @@
         <v>28</v>
       </c>
     </row>
-    <row r="53" spans="1:50" ht="36" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A53" s="12" t="s">
-        <v>52</v>
-      </c>
-      <c r="B53" s="8">
+    <row r="53" spans="1:50" ht="36" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A53" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B53" s="7">
         <v>28</v>
       </c>
-      <c r="C53" s="9">
+      <c r="C53" s="8">
         <v>33</v>
       </c>
-      <c r="D53" s="8">
+      <c r="D53" s="7">
         <v>40</v>
       </c>
-      <c r="E53" s="8">
+      <c r="E53" s="7">
         <v>22</v>
       </c>
-      <c r="F53" s="8">
+      <c r="F53" s="7">
         <v>12</v>
       </c>
-      <c r="G53" s="8">
+      <c r="G53" s="7">
         <v>24</v>
       </c>
-      <c r="H53" s="8">
+      <c r="H53" s="7">
         <v>12</v>
       </c>
-      <c r="I53" s="8">
+      <c r="I53" s="7">
         <v>33</v>
       </c>
-      <c r="J53" s="8">
+      <c r="J53" s="7">
         <v>12</v>
       </c>
-      <c r="K53" s="8">
+      <c r="K53" s="7">
         <v>27</v>
       </c>
-      <c r="L53" s="8">
+      <c r="L53" s="7">
         <v>14</v>
       </c>
-      <c r="M53" s="8">
+      <c r="M53" s="7">
         <v>24</v>
       </c>
-      <c r="N53" s="8">
+      <c r="N53" s="7">
         <v>20</v>
       </c>
-      <c r="O53" s="9">
+      <c r="O53" s="8">
         <v>16</v>
       </c>
-      <c r="P53" s="8">
+      <c r="P53" s="7">
         <v>15</v>
       </c>
-      <c r="Q53" s="9">
+      <c r="Q53" s="8">
         <v>21</v>
       </c>
-      <c r="R53" s="8">
+      <c r="R53" s="7">
         <v>65</v>
       </c>
-      <c r="S53" s="8">
+      <c r="S53" s="7">
         <v>39</v>
       </c>
-      <c r="T53" s="8">
+      <c r="T53" s="7">
         <v>10</v>
       </c>
-      <c r="U53" s="8">
+      <c r="U53" s="7">
         <v>27</v>
       </c>
-      <c r="V53" s="8">
+      <c r="V53" s="7">
         <v>21</v>
       </c>
-      <c r="W53" s="8">
+      <c r="W53" s="7">
         <v>22</v>
       </c>
-      <c r="X53" s="8">
+      <c r="X53" s="7">
         <v>32</v>
       </c>
-      <c r="Y53" s="8">
+      <c r="Y53" s="7">
         <v>23</v>
       </c>
-      <c r="Z53" s="8">
+      <c r="Z53" s="7">
         <v>26</v>
       </c>
-      <c r="AA53" s="8">
+      <c r="AA53" s="7">
         <v>22</v>
       </c>
-      <c r="AB53" s="8">
+      <c r="AB53" s="7">
         <v>22</v>
       </c>
-      <c r="AC53" s="8">
+      <c r="AC53" s="7">
         <v>17</v>
       </c>
-      <c r="AD53" s="8">
+      <c r="AD53" s="7">
         <v>34</v>
       </c>
-      <c r="AE53" s="8">
+      <c r="AE53" s="7">
         <v>11</v>
       </c>
-      <c r="AF53" s="8">
+      <c r="AF53" s="7">
         <v>21</v>
       </c>
-      <c r="AG53" s="9">
+      <c r="AG53" s="8">
         <v>28</v>
       </c>
-      <c r="AH53" s="8">
+      <c r="AH53" s="7">
         <v>38</v>
       </c>
-      <c r="AI53" s="8">
+      <c r="AI53" s="7">
         <v>12</v>
       </c>
-      <c r="AJ53" s="8">
+      <c r="AJ53" s="7">
         <v>10</v>
       </c>
-      <c r="AK53" s="8">
+      <c r="AK53" s="7">
         <v>28</v>
       </c>
-      <c r="AL53" s="8">
+      <c r="AL53" s="7">
         <v>16</v>
       </c>
-      <c r="AM53" s="8">
+      <c r="AM53" s="7">
         <v>11</v>
       </c>
-      <c r="AN53" s="8">
+      <c r="AN53" s="7">
         <v>17</v>
       </c>
-      <c r="AO53" s="8">
+      <c r="AO53" s="7">
         <v>22</v>
       </c>
-      <c r="AP53" s="8">
+      <c r="AP53" s="7">
         <v>13</v>
       </c>
-      <c r="AQ53" s="8">
+      <c r="AQ53" s="7">
         <v>10</v>
       </c>
-      <c r="AR53" s="8">
+      <c r="AR53" s="7">
         <v>21</v>
       </c>
-      <c r="AS53" s="8">
+      <c r="AS53" s="7">
         <v>25</v>
       </c>
-      <c r="AT53" s="8">
+      <c r="AT53" s="7">
         <v>22</v>
       </c>
-      <c r="AU53" s="8">
+      <c r="AU53" s="7">
         <v>67</v>
       </c>
-      <c r="AV53" s="8">
+      <c r="AV53" s="7">
         <v>55</v>
       </c>
-      <c r="AW53" s="8">
+      <c r="AW53" s="7">
         <v>28</v>
       </c>
       <c r="AX53">
@@ -8682,12 +8517,12 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9FC8517F-B0FA-4B90-91DA-AA356DB0AF81}">
   <dimension ref="A1:AW52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="25.44140625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="25.42578125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>48</v>
       </c>
@@ -8836,7 +8671,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -8985,7 +8820,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
@@ -9134,7 +8969,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
@@ -9283,7 +9118,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -9432,7 +9267,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
@@ -9581,7 +9416,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -9730,7 +9565,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>11</v>
       </c>
@@ -9879,7 +9714,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -10028,7 +9863,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>13</v>
       </c>
@@ -10177,7 +10012,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
@@ -10326,7 +10161,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>0</v>
       </c>
@@ -10475,7 +10310,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>15</v>
       </c>
@@ -10624,7 +10459,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
@@ -10773,7 +10608,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
@@ -10922,7 +10757,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>18</v>
       </c>
@@ -11071,7 +10906,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
@@ -11220,7 +11055,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
@@ -11369,7 +11204,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>21</v>
       </c>
@@ -11518,7 +11353,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="20" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>22</v>
       </c>
@@ -11667,7 +11502,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>23</v>
       </c>
@@ -11816,7 +11651,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="22" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>24</v>
       </c>
@@ -11965,7 +11800,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>25</v>
       </c>
@@ -12114,7 +11949,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
@@ -12263,7 +12098,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="25" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>27</v>
       </c>
@@ -12412,7 +12247,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="26" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>28</v>
       </c>
@@ -12561,7 +12396,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="27" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>1</v>
       </c>
@@ -12710,7 +12545,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>29</v>
       </c>
@@ -12859,7 +12694,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>30</v>
       </c>
@@ -13008,7 +12843,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
@@ -13157,7 +12992,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="31" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>32</v>
       </c>
@@ -13306,7 +13141,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="32" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>33</v>
       </c>
@@ -13455,7 +13290,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>34</v>
       </c>
@@ -13604,7 +13439,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="34" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>35</v>
       </c>
@@ -13753,7 +13588,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>36</v>
       </c>
@@ -13902,7 +13737,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>37</v>
       </c>
@@ -14051,7 +13886,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="37" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>2</v>
       </c>
@@ -14200,7 +14035,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="38" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>38</v>
       </c>
@@ -14349,7 +14184,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="39" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>39</v>
       </c>
@@ -14498,7 +14333,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="40" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>40</v>
       </c>
@@ -14647,7 +14482,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="41" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>41</v>
       </c>
@@ -14796,7 +14631,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="42" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>42</v>
       </c>
@@ -14945,7 +14780,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>43</v>
       </c>
@@ -15094,7 +14929,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="44" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>3</v>
       </c>
@@ -15243,7 +15078,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="45" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>44</v>
       </c>
@@ -15392,7 +15227,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="46" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>45</v>
       </c>
@@ -15541,7 +15376,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>46</v>
       </c>
@@ -15690,7 +15525,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>4</v>
       </c>
@@ -15839,7 +15674,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>47</v>
       </c>
@@ -15988,152 +15823,152 @@
         <v>4</v>
       </c>
     </row>
-    <row r="52" spans="1:49" ht="41.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B52" s="8">
+    <row r="52" spans="1:49" ht="41.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52" s="7">
         <v>5</v>
       </c>
-      <c r="C52" s="8">
-        <v>0</v>
-      </c>
-      <c r="D52" s="8">
+      <c r="C52" s="7">
+        <v>0</v>
+      </c>
+      <c r="D52" s="7">
         <v>7</v>
       </c>
-      <c r="E52" s="8">
+      <c r="E52" s="7">
         <v>8</v>
       </c>
-      <c r="F52" s="8">
-        <v>2</v>
-      </c>
-      <c r="G52" s="8">
+      <c r="F52" s="7">
+        <v>2</v>
+      </c>
+      <c r="G52" s="7">
         <v>10</v>
       </c>
-      <c r="H52" s="8">
+      <c r="H52" s="7">
         <v>5</v>
       </c>
-      <c r="I52" s="8">
+      <c r="I52" s="7">
         <v>14</v>
       </c>
-      <c r="J52" s="8">
+      <c r="J52" s="7">
         <v>7</v>
       </c>
-      <c r="K52" s="8">
+      <c r="K52" s="7">
         <v>5</v>
       </c>
-      <c r="L52" s="8">
-        <v>2</v>
-      </c>
-      <c r="M52" s="9">
+      <c r="L52" s="7">
+        <v>2</v>
+      </c>
+      <c r="M52" s="8">
         <v>5</v>
       </c>
-      <c r="N52" s="8">
+      <c r="N52" s="7">
         <v>6</v>
       </c>
-      <c r="O52" s="8">
-        <v>0</v>
-      </c>
-      <c r="P52" s="8">
+      <c r="O52" s="7">
+        <v>0</v>
+      </c>
+      <c r="P52" s="7">
         <v>5</v>
       </c>
-      <c r="Q52" s="9">
+      <c r="Q52" s="8">
         <v>11</v>
       </c>
-      <c r="R52" s="8">
+      <c r="R52" s="7">
         <v>31</v>
       </c>
-      <c r="S52" s="8">
+      <c r="S52" s="7">
         <v>10</v>
       </c>
-      <c r="T52" s="8">
+      <c r="T52" s="7">
         <v>6</v>
       </c>
-      <c r="U52" s="8">
+      <c r="U52" s="7">
         <v>9</v>
       </c>
-      <c r="V52" s="9">
+      <c r="V52" s="8">
         <v>7</v>
       </c>
-      <c r="W52" s="8">
+      <c r="W52" s="7">
         <v>7</v>
       </c>
-      <c r="X52" s="8">
+      <c r="X52" s="7">
         <v>11</v>
       </c>
-      <c r="Y52" s="8">
+      <c r="Y52" s="7">
         <v>7</v>
       </c>
-      <c r="Z52" s="8">
+      <c r="Z52" s="7">
         <v>10</v>
       </c>
-      <c r="AA52" s="8">
+      <c r="AA52" s="7">
         <v>8</v>
       </c>
-      <c r="AB52" s="8">
+      <c r="AB52" s="7">
         <v>14</v>
       </c>
-      <c r="AC52" s="8">
+      <c r="AC52" s="7">
         <v>5</v>
       </c>
-      <c r="AD52" s="8">
+      <c r="AD52" s="7">
         <v>13</v>
       </c>
-      <c r="AE52" s="8">
-        <v>2</v>
-      </c>
-      <c r="AF52" s="8">
+      <c r="AE52" s="7">
+        <v>2</v>
+      </c>
+      <c r="AF52" s="7">
         <v>7</v>
       </c>
-      <c r="AG52" s="8">
+      <c r="AG52" s="7">
         <v>7</v>
       </c>
-      <c r="AH52" s="8">
+      <c r="AH52" s="7">
         <v>18</v>
       </c>
-      <c r="AI52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AJ52" s="8">
+      <c r="AI52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AJ52" s="7">
         <v>5</v>
       </c>
-      <c r="AK52" s="8">
+      <c r="AK52" s="7">
         <v>4</v>
       </c>
-      <c r="AL52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AM52" s="8">
+      <c r="AL52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AM52" s="7">
         <v>7</v>
       </c>
-      <c r="AN52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AO52" s="8">
+      <c r="AN52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AO52" s="7">
         <v>9</v>
       </c>
-      <c r="AP52" s="8">
+      <c r="AP52" s="7">
         <v>5</v>
       </c>
-      <c r="AQ52" s="8">
-        <v>1</v>
-      </c>
-      <c r="AR52" s="8">
+      <c r="AQ52" s="7">
+        <v>1</v>
+      </c>
+      <c r="AR52" s="7">
         <v>5</v>
       </c>
-      <c r="AS52" s="8">
+      <c r="AS52" s="7">
         <v>8</v>
       </c>
-      <c r="AT52" s="8">
+      <c r="AT52" s="7">
         <v>10</v>
       </c>
-      <c r="AU52" s="8">
+      <c r="AU52" s="7">
         <v>24</v>
       </c>
-      <c r="AV52" s="8">
+      <c r="AV52" s="7">
         <v>20</v>
       </c>
-      <c r="AW52" s="8">
+      <c r="AW52" s="7">
         <v>4</v>
       </c>
     </row>
@@ -16145,12 +15980,12 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2C9856D8-0D73-4336-AC8A-142F2E0F58A4}">
   <dimension ref="A1:AW52"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="28.44140625" style="6" customWidth="1"/>
+    <col min="1" max="1" width="28.42578125" style="6" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:49" s="6" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:49" s="6" customFormat="1" x14ac:dyDescent="0.25">
       <c r="A1" s="5" t="s">
         <v>48</v>
       </c>
@@ -16299,7 +16134,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="2" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>5</v>
       </c>
@@ -16448,7 +16283,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A3" s="5" t="s">
         <v>6</v>
       </c>
@@ -16597,7 +16432,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="4" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A4" s="5" t="s">
         <v>7</v>
       </c>
@@ -16746,7 +16581,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="5" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A5" s="5" t="s">
         <v>8</v>
       </c>
@@ -16895,7 +16730,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A6" s="5" t="s">
         <v>9</v>
       </c>
@@ -17044,7 +16879,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A7" s="5" t="s">
         <v>10</v>
       </c>
@@ -17193,7 +17028,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="8" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A8" s="5" t="s">
         <v>11</v>
       </c>
@@ -17342,7 +17177,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A9" s="5" t="s">
         <v>12</v>
       </c>
@@ -17491,7 +17326,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="10" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A10" s="5" t="s">
         <v>13</v>
       </c>
@@ -17640,7 +17475,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A11" s="5" t="s">
         <v>14</v>
       </c>
@@ -17789,7 +17624,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="12" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A12" s="5" t="s">
         <v>0</v>
       </c>
@@ -17938,7 +17773,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="13" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A13" s="5" t="s">
         <v>15</v>
       </c>
@@ -18087,7 +17922,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A14" s="5" t="s">
         <v>16</v>
       </c>
@@ -18236,7 +18071,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A15" s="5" t="s">
         <v>17</v>
       </c>
@@ -18385,7 +18220,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A16" s="5" t="s">
         <v>18</v>
       </c>
@@ -18534,7 +18369,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A17" s="5" t="s">
         <v>19</v>
       </c>
@@ -18683,7 +18518,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A18" s="5" t="s">
         <v>20</v>
       </c>
@@ -18832,7 +18667,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="19" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A19" s="5" t="s">
         <v>21</v>
       </c>
@@ -18981,7 +18816,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A20" s="5" t="s">
         <v>22</v>
       </c>
@@ -19130,7 +18965,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A21" s="5" t="s">
         <v>23</v>
       </c>
@@ -19279,7 +19114,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="22" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A22" s="5" t="s">
         <v>24</v>
       </c>
@@ -19428,7 +19263,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A23" s="5" t="s">
         <v>25</v>
       </c>
@@ -19577,7 +19412,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="24" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A24" s="5" t="s">
         <v>26</v>
       </c>
@@ -19726,7 +19561,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="25" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A25" s="5" t="s">
         <v>27</v>
       </c>
@@ -19875,7 +19710,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A26" s="5" t="s">
         <v>28</v>
       </c>
@@ -20024,7 +19859,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A27" s="5" t="s">
         <v>1</v>
       </c>
@@ -20173,7 +20008,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A28" s="5" t="s">
         <v>29</v>
       </c>
@@ -20322,7 +20157,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="29" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A29" s="5" t="s">
         <v>30</v>
       </c>
@@ -20471,7 +20306,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A30" s="5" t="s">
         <v>31</v>
       </c>
@@ -20620,7 +20455,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="31" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A31" s="5" t="s">
         <v>32</v>
       </c>
@@ -20769,7 +20604,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="32" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A32" s="5" t="s">
         <v>33</v>
       </c>
@@ -20918,7 +20753,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="33" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A33" s="5" t="s">
         <v>34</v>
       </c>
@@ -21067,7 +20902,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="34" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A34" s="5" t="s">
         <v>35</v>
       </c>
@@ -21216,7 +21051,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="35" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A35" s="5" t="s">
         <v>36</v>
       </c>
@@ -21365,7 +21200,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="36" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A36" s="5" t="s">
         <v>37</v>
       </c>
@@ -21514,7 +21349,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="37" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A37" s="5" t="s">
         <v>2</v>
       </c>
@@ -21663,7 +21498,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="38" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A38" s="5" t="s">
         <v>38</v>
       </c>
@@ -21812,7 +21647,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="39" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A39" s="5" t="s">
         <v>39</v>
       </c>
@@ -21961,7 +21796,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="40" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A40" s="5" t="s">
         <v>40</v>
       </c>
@@ -22110,7 +21945,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="41" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A41" s="5" t="s">
         <v>41</v>
       </c>
@@ -22259,7 +22094,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="42" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A42" s="5" t="s">
         <v>42</v>
       </c>
@@ -22408,7 +22243,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="43" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A43" s="5" t="s">
         <v>43</v>
       </c>
@@ -22557,7 +22392,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A44" s="5" t="s">
         <v>3</v>
       </c>
@@ -22706,7 +22541,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A45" s="5" t="s">
         <v>44</v>
       </c>
@@ -22855,7 +22690,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="46" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A46" s="5" t="s">
         <v>45</v>
       </c>
@@ -23004,7 +22839,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A47" s="5" t="s">
         <v>46</v>
       </c>
@@ -23153,7 +22988,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="48" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A48" s="5" t="s">
         <v>4</v>
       </c>
@@ -23302,7 +23137,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:49" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:49" x14ac:dyDescent="0.25">
       <c r="A49" s="5" t="s">
         <v>47</v>
       </c>
@@ -23451,152 +23286,152 @@
         <v>16</v>
       </c>
     </row>
-    <row r="52" spans="1:49" s="12" customFormat="1" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A52" s="13" t="s">
-        <v>52</v>
-      </c>
-      <c r="B52" s="8">
+    <row r="52" spans="1:49" s="10" customFormat="1" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A52" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="B52" s="7">
         <v>9</v>
       </c>
-      <c r="C52" s="8">
+      <c r="C52" s="7">
         <v>13</v>
       </c>
-      <c r="D52" s="8">
+      <c r="D52" s="7">
         <v>14</v>
       </c>
-      <c r="E52" s="8">
+      <c r="E52" s="7">
         <v>7</v>
       </c>
-      <c r="F52" s="8">
+      <c r="F52" s="7">
         <v>8</v>
       </c>
-      <c r="G52" s="8">
+      <c r="G52" s="7">
         <v>6</v>
       </c>
-      <c r="H52" s="8">
-        <v>0</v>
-      </c>
-      <c r="I52" s="8">
+      <c r="H52" s="7">
+        <v>0</v>
+      </c>
+      <c r="I52" s="7">
         <v>6</v>
       </c>
-      <c r="J52" s="8">
-        <v>1</v>
-      </c>
-      <c r="K52" s="8">
+      <c r="J52" s="7">
+        <v>1</v>
+      </c>
+      <c r="K52" s="7">
         <v>9</v>
       </c>
-      <c r="L52" s="8">
+      <c r="L52" s="7">
         <v>8</v>
       </c>
-      <c r="M52" s="8">
-        <v>2</v>
-      </c>
-      <c r="N52" s="8">
-        <v>2</v>
-      </c>
-      <c r="O52" s="9">
+      <c r="M52" s="7">
+        <v>2</v>
+      </c>
+      <c r="N52" s="7">
+        <v>2</v>
+      </c>
+      <c r="O52" s="8">
         <v>7</v>
       </c>
-      <c r="P52" s="8">
-        <v>1</v>
-      </c>
-      <c r="Q52" s="8">
-        <v>3</v>
-      </c>
-      <c r="R52" s="8">
+      <c r="P52" s="7">
+        <v>1</v>
+      </c>
+      <c r="Q52" s="7">
+        <v>3</v>
+      </c>
+      <c r="R52" s="7">
         <v>7</v>
       </c>
-      <c r="S52" s="8">
+      <c r="S52" s="7">
         <v>8</v>
       </c>
-      <c r="T52" s="8">
-        <v>0</v>
-      </c>
-      <c r="U52" s="8">
+      <c r="T52" s="7">
+        <v>0</v>
+      </c>
+      <c r="U52" s="7">
         <v>7</v>
       </c>
-      <c r="V52" s="8">
+      <c r="V52" s="7">
         <v>4</v>
       </c>
-      <c r="W52" s="8">
+      <c r="W52" s="7">
         <v>6</v>
       </c>
-      <c r="X52" s="8">
+      <c r="X52" s="7">
         <v>8</v>
       </c>
-      <c r="Y52" s="8">
+      <c r="Y52" s="7">
         <v>6</v>
       </c>
-      <c r="Z52" s="8">
+      <c r="Z52" s="7">
         <v>7</v>
       </c>
-      <c r="AA52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AB52" s="8">
-        <v>2</v>
-      </c>
-      <c r="AC52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AD52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AE52" s="8">
-        <v>1</v>
-      </c>
-      <c r="AF52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AG52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AH52" s="8">
-        <v>0</v>
-      </c>
-      <c r="AI52" s="8">
-        <v>1</v>
-      </c>
-      <c r="AJ52" s="8">
-        <v>2</v>
-      </c>
-      <c r="AK52" s="8">
+      <c r="AA52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AB52" s="7">
+        <v>2</v>
+      </c>
+      <c r="AC52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AD52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AE52" s="7">
+        <v>1</v>
+      </c>
+      <c r="AF52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AG52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AH52" s="7">
+        <v>0</v>
+      </c>
+      <c r="AI52" s="7">
+        <v>1</v>
+      </c>
+      <c r="AJ52" s="7">
+        <v>2</v>
+      </c>
+      <c r="AK52" s="7">
         <v>6</v>
       </c>
-      <c r="AL52" s="8">
-        <v>1</v>
-      </c>
-      <c r="AM52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AN52" s="8">
-        <v>1</v>
-      </c>
-      <c r="AO52" s="8">
-        <v>2</v>
-      </c>
-      <c r="AP52" s="8">
-        <v>0</v>
-      </c>
-      <c r="AQ52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AR52" s="8">
-        <v>3</v>
-      </c>
-      <c r="AS52" s="8">
-        <v>2</v>
-      </c>
-      <c r="AT52" s="8">
-        <v>2</v>
-      </c>
-      <c r="AU52" s="8">
+      <c r="AL52" s="7">
+        <v>1</v>
+      </c>
+      <c r="AM52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AN52" s="7">
+        <v>1</v>
+      </c>
+      <c r="AO52" s="7">
+        <v>2</v>
+      </c>
+      <c r="AP52" s="7">
+        <v>0</v>
+      </c>
+      <c r="AQ52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AR52" s="7">
+        <v>3</v>
+      </c>
+      <c r="AS52" s="7">
+        <v>2</v>
+      </c>
+      <c r="AT52" s="7">
+        <v>2</v>
+      </c>
+      <c r="AU52" s="7">
         <v>5</v>
       </c>
-      <c r="AV52" s="8">
+      <c r="AV52" s="7">
         <v>10</v>
       </c>
-      <c r="AW52" s="8">
+      <c r="AW52" s="7">
         <v>16</v>
       </c>
     </row>

</xml_diff>